<commit_message>
Fix Excel R&B and AMC report quality: mappings, photos, red fills, Column J
- R&B Appendix-A: remove all hardcoded defaults/fallbacks; map date_of_completion,
  date_of_survey, surface_utilities, performance correctly; blank when no user data
- R&B Appendix-B: full rewrite covering all sections 1–19 + row 128; fix off-by-one
  in sections 5/6/7; add sections 11–19 (expansion joints through maintenance history);
  section 20 (maintenance recommendations) intentionally left blank
- Remove Column J from R&B Appendix-B entirely: deleted from template XML and code
- AMC Appendix-A: remove red row fills from rows 58, 84, 92–94 in template
- R&B Appendix-A: remove red row fills from rows 58, 84, 92–94 in template
- Both formats: fix photo upscaling — images now only downscale, never stretch up

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/casad_amc_template.xlsx
+++ b/casad_amc_template.xlsx
@@ -3853,7 +3853,7 @@
       </c>
       <c r="D57" s="241" t="n"/>
     </row>
-    <row r="58" ht="38.25" customFormat="1" customHeight="1" s="4">
+    <row r="58" ht="38.25" customHeight="1">
       <c r="A58" s="246" t="n"/>
       <c r="B58" s="127" t="inlineStr">
         <is>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="D83" s="241" t="n"/>
     </row>
-    <row r="84" ht="51" customFormat="1" customHeight="1" s="5">
+    <row r="84" ht="51" customHeight="1">
       <c r="A84" s="162" t="inlineStr">
         <is>
           <t>(e)</t>
@@ -4409,7 +4409,7 @@
       </c>
       <c r="D91" s="241" t="n"/>
     </row>
-    <row r="92" ht="39.75" customFormat="1" customHeight="1" s="5">
+    <row r="92" ht="39.75" customHeight="1">
       <c r="A92" s="124" t="n">
         <v>8</v>
       </c>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="D92" s="241" t="n"/>
     </row>
-    <row r="93" ht="24" customFormat="1" customHeight="1" s="5">
+    <row r="93" ht="24" customHeight="1">
       <c r="A93" s="124" t="n">
         <v>9</v>
       </c>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="D93" s="241" t="n"/>
     </row>
-    <row r="94" ht="25.5" customFormat="1" customHeight="1" s="5">
+    <row r="94" ht="25.5" customHeight="1">
       <c r="A94" s="124" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Fix Section 4 subsoil template split cells + strengthen unit normalization
- casad_amc_template.xlsx: merge C:D for rows 33-39 (Sub Soil Particulars section
  header + rows a-f). Previously C and D were separate cells both showing 'Not
  Available', causing a split-column appearance. Now each row has one merged
  answer cell, matching all other Appendix-A rows.
- ai_parse.py: promote unit/operator normalization from a weak EXCEPTION sub-bullet
  to a top-level ALWAYS APPLY rule. Ensures 'meter' → 'm' and 'plus' → '+' are
  applied to ALL fields including carriage_width and footpath_width, regardless of
  the copy-exactly rule.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/casad_amc_template.xlsx
+++ b/casad_amc_template.xlsx
@@ -3442,11 +3442,6 @@
           <t xml:space="preserve">Data Not Available </t>
         </is>
       </c>
-      <c r="D33" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="162" t="inlineStr">
@@ -3464,11 +3459,6 @@
           <t xml:space="preserve">Not Available </t>
         </is>
       </c>
-      <c r="D34" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="162" t="inlineStr">
@@ -3486,11 +3476,6 @@
           <t xml:space="preserve">Not Available </t>
         </is>
       </c>
-      <c r="D35" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="162" t="inlineStr">
@@ -3508,11 +3493,6 @@
           <t xml:space="preserve">Not Available </t>
         </is>
       </c>
-      <c r="D36" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="162" t="inlineStr">
@@ -3530,11 +3510,6 @@
           <t xml:space="preserve">Not Available </t>
         </is>
       </c>
-      <c r="D37" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="162" t="inlineStr">
@@ -3552,11 +3527,6 @@
           <t xml:space="preserve">Not Available </t>
         </is>
       </c>
-      <c r="D38" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="162" t="inlineStr">
@@ -3570,11 +3540,6 @@
         </is>
       </c>
       <c r="C39" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Available </t>
-        </is>
-      </c>
-      <c r="D39" s="103" t="inlineStr">
         <is>
           <t xml:space="preserve">Not Available </t>
         </is>
@@ -4579,7 +4544,7 @@
       <c r="D109" s="111" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="90">
+  <mergeCells count="97">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C62:D62"/>
     <mergeCell ref="C15:D15"/>
@@ -4670,6 +4635,13 @@
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C78:D78"/>
     <mergeCell ref="C87:D87"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7086614173228347" right="0.4724409448818898" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>

</xml_diff>